<commit_message>
Sync website content 2026-05-20 16:57
</commit_message>
<xml_diff>
--- a/组合介绍/report_assets/main/workbooks/1-Microsoft_Excel_Worksheet1.xlsx
+++ b/组合介绍/report_assets/main/workbooks/1-Microsoft_Excel_Worksheet1.xlsx
@@ -125,14 +125,14 @@
     <xf applyAlignment="false" applyBorder="false" applyFill="false" applyFont="false" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="true" applyProtection="false" borderId="1" fillId="0" fontId="1" numFmtId="164" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="true" applyProtection="false" borderId="3" fillId="0" fontId="1" numFmtId="164" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="3" fillId="0" fontId="1" numFmtId="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -458,7 +458,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1"/>
+      <c r="A1" s="3"/>
       <c r="B1" s="2" t="str">
         <v>年化收益率</v>
       </c>
@@ -476,16 +476,16 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="str">
+      <c r="A2" s="3" t="str">
         <v>普林格策略(70/30)</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="1">
         <v>0.1056</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="1">
         <v>-0.1432</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="1">
         <v>0.1074</v>
       </c>
       <c r="E2" s="2">
@@ -496,16 +496,16 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="str">
+      <c r="A3" s="3" t="str">
         <v>沪深300(基准)</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="1">
         <v>0.0532</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="1">
         <v>-0.4156</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="1">
         <v>0.182</v>
       </c>
       <c r="E3" s="2">

</xml_diff>